<commit_message>
adding api and some changes to extraction
</commit_message>
<xml_diff>
--- a/FichiersClaude/comparaison_EBA/Comparaison_EBA_vs_resultats_2025-12-31.xlsx
+++ b/FichiersClaude/comparaison_EBA/Comparaison_EBA_vs_resultats_2025-12-31.xlsx
@@ -600,17 +600,17 @@
         <v>0.0512</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0225</v>
+        <v>0.0512</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0287</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>127.5555555555556</v>
+        <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1946,23 +1946,17 @@
       <c r="D44" t="n">
         <v>0.2079427881739253</v>
       </c>
-      <c r="E44" t="n">
-        <v>0.208</v>
-      </c>
-      <c r="F44" t="n">
-        <v>-5.721182607468234e-05</v>
-      </c>
-      <c r="G44" t="n">
-        <v>-0.02750568561282804</v>
-      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>page 148 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -2129,23 +2123,17 @@
       <c r="D49" t="n">
         <v>1.0701</v>
       </c>
-      <c r="E49" t="n">
-        <v>103.5</v>
-      </c>
-      <c r="F49" t="n">
-        <v>-102.4299</v>
-      </c>
-      <c r="G49" t="n">
-        <v>-98.96608695652174</v>
-      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>ANOMALIE UNITE PROBABLE (facteur ~100, fichier resultats)</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>page 104 (Qwen2.5-VL)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -2400,19 +2388,17 @@
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
-      <c r="E56" t="n">
-        <v>37812211</v>
-      </c>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Absent du fichier resultats</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>page 149 (Qwen2.5-VL)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -2667,19 +2653,17 @@
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
-      <c r="E63" t="n">
-        <v>1.0829</v>
-      </c>
+      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Absent du fichier resultats</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>page 8 (OCR table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -2859,13 +2843,13 @@
         <v>566950024783.033</v>
       </c>
       <c r="E68" t="n">
-        <v>420000000</v>
+        <v>595000000</v>
       </c>
       <c r="F68" t="n">
-        <v>566530024783.033</v>
+        <v>566355024783.033</v>
       </c>
       <c r="G68" t="n">
-        <v>134888.1011388174</v>
+        <v>95185.71845092991</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -2874,7 +2858,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>page 1 (OCR table)</t>
+          <t>page 2 (OCR table)</t>
         </is>
       </c>
     </row>
@@ -2897,23 +2881,17 @@
       <c r="D69" t="n">
         <v>40175045947.4999</v>
       </c>
-      <c r="E69" t="n">
-        <v>526000000</v>
-      </c>
-      <c r="F69" t="n">
-        <v>39649045947.4999</v>
-      </c>
-      <c r="G69" t="n">
-        <v>7537.841434885912</v>
-      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>page 2 (OCR table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -2976,13 +2954,13 @@
         <v>112475232762.5</v>
       </c>
       <c r="E71" t="n">
-        <v>586000000</v>
+        <v>1000000</v>
       </c>
       <c r="F71" t="n">
-        <v>111889232762.5</v>
+        <v>112474232762.5</v>
       </c>
       <c r="G71" t="n">
-        <v>19093.72572738908</v>
+        <v>11247423.27625</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -2991,7 +2969,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>page 2 (OCR table)</t>
+          <t>page 3 (OCR table)</t>
         </is>
       </c>
     </row>
@@ -3177,19 +3155,17 @@
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
-      <c r="E77" t="n">
-        <v>1.0829</v>
-      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Absent du fichier resultats</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>page 8 (OCR table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3319,7 @@
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="n">
-        <v>420000000</v>
+        <v>595000000</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
@@ -3354,7 +3330,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>page 1 (OCR table)</t>
+          <t>page 2 (OCR table)</t>
         </is>
       </c>
     </row>
@@ -3375,19 +3351,17 @@
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
-      <c r="E83" t="n">
-        <v>526000000</v>
-      </c>
+      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Absent du fichier resultats</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>page 2 (OCR table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -3442,7 +3416,7 @@
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="n">
-        <v>586000000</v>
+        <v>1000000</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
@@ -3453,7 +3427,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>page 2 (OCR table)</t>
+          <t>page 3 (OCR table)</t>
         </is>
       </c>
     </row>
@@ -3515,23 +3489,17 @@
       <c r="D87" t="n">
         <v>0.1798597690275607</v>
       </c>
-      <c r="E87" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="F87" t="n">
-        <v>-0.0001402309724393425</v>
-      </c>
-      <c r="G87" t="n">
-        <v>-0.0779060957996347</v>
-      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>page 17 (Qwen2.5-VL)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -4136,23 +4104,17 @@
       <c r="D104" t="n">
         <v>1.4499</v>
       </c>
-      <c r="E104" t="n">
-        <v>1</v>
-      </c>
-      <c r="F104" t="n">
-        <v>0.4499</v>
-      </c>
-      <c r="G104" t="n">
-        <v>44.98999999999999</v>
-      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>page 118 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5059,13 +5021,13 @@
         <v>1.3512</v>
       </c>
       <c r="E132" t="n">
-        <v>1</v>
+        <v>8.52</v>
       </c>
       <c r="F132" t="n">
-        <v>0.3512</v>
+        <v>-7.168799999999999</v>
       </c>
       <c r="G132" t="n">
-        <v>35.12</v>
+        <v>-84.14084507042253</v>
       </c>
       <c r="H132" t="inlineStr">
         <is>
@@ -5074,7 +5036,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>page 100 (table)</t>
+          <t>page 101 (table)</t>
         </is>
       </c>
     </row>
@@ -5411,7 +5373,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -5422,23 +5384,17 @@
       <c r="D142" t="n">
         <v>0.2099646719607195</v>
       </c>
-      <c r="E142" t="n">
-        <v>0.154</v>
-      </c>
-      <c r="F142" t="n">
-        <v>0.05596467196071947</v>
-      </c>
-      <c r="G142" t="n">
-        <v>36.34069607838926</v>
-      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>page 9 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5450,7 +5406,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -5461,23 +5417,17 @@
       <c r="D143" t="n">
         <v>0.2099646719607195</v>
       </c>
-      <c r="E143" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="F143" t="n">
-        <v>0.03196467196071945</v>
-      </c>
-      <c r="G143" t="n">
-        <v>17.95768087680868</v>
-      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>page 10 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5439,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -5500,23 +5450,17 @@
       <c r="D144" t="n">
         <v>0.2417087285470789</v>
       </c>
-      <c r="E144" t="n">
-        <v>0.209</v>
-      </c>
-      <c r="F144" t="n">
-        <v>0.03270872854707887</v>
-      </c>
-      <c r="G144" t="n">
-        <v>15.65010935266932</v>
-      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>page 10 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5472,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -5539,23 +5483,17 @@
       <c r="D145" t="n">
         <v>0.08173300507627101</v>
       </c>
-      <c r="E145" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="F145" t="n">
-        <v>0.02873300507627102</v>
-      </c>
-      <c r="G145" t="n">
-        <v>54.21321712503966</v>
-      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>page 9 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5567,7 +5505,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -5578,23 +5516,17 @@
       <c r="D146" t="n">
         <v>2.431033333333334</v>
       </c>
-      <c r="E146" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="F146" t="n">
-        <v>0.9010333333333336</v>
-      </c>
-      <c r="G146" t="n">
-        <v>58.89106753812637</v>
-      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>page 9 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5606,7 +5538,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -5617,23 +5549,17 @@
       <c r="D147" t="n">
         <v>1.2608028</v>
       </c>
-      <c r="E147" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="F147" t="n">
-        <v>-0.1491971999999999</v>
-      </c>
-      <c r="G147" t="n">
-        <v>-10.58136170212765</v>
-      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>page 9 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5645,7 +5571,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -5656,23 +5582,17 @@
       <c r="D148" t="n">
         <v>8864214631.894703</v>
       </c>
-      <c r="E148" t="n">
-        <v>20900000</v>
-      </c>
-      <c r="F148" t="n">
-        <v>8843314631.894703</v>
-      </c>
-      <c r="G148" t="n">
-        <v>42312.51020045312</v>
-      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>page 9 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5684,7 +5604,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -5695,23 +5615,17 @@
       <c r="D149" t="n">
         <v>8864214631.894703</v>
       </c>
-      <c r="E149" t="n">
-        <v>24127000000</v>
-      </c>
-      <c r="F149" t="n">
-        <v>-15262785368.1053</v>
-      </c>
-      <c r="G149" t="n">
-        <v>-63.26018720978694</v>
-      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>page 10 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5637,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -5734,23 +5648,17 @@
       <c r="D150" t="n">
         <v>10204374041.76505</v>
       </c>
-      <c r="E150" t="n">
-        <v>28241000000</v>
-      </c>
-      <c r="F150" t="n">
-        <v>-18036625958.23495</v>
-      </c>
-      <c r="G150" t="n">
-        <v>-63.86681051745671</v>
-      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>page 10 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5762,7 +5670,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -5773,23 +5681,17 @@
       <c r="D151" t="n">
         <v>42217648088.6891</v>
       </c>
-      <c r="E151" t="n">
-        <v>135398000000</v>
-      </c>
-      <c r="F151" t="n">
-        <v>-93180351911.3109</v>
-      </c>
-      <c r="G151" t="n">
-        <v>-68.8195925429555</v>
-      </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>page 10 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5703,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -5812,23 +5714,17 @@
       <c r="D152" t="n">
         <v>1521669142.132596</v>
       </c>
-      <c r="E152" t="n">
-        <v>108376000000</v>
-      </c>
-      <c r="F152" t="n">
-        <v>-106854330857.8674</v>
-      </c>
-      <c r="G152" t="n">
-        <v>-98.59593531581476</v>
-      </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>page 15 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5840,7 +5736,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -5851,23 +5747,17 @@
       <c r="D153" t="n">
         <v>18300108182.78608</v>
       </c>
-      <c r="E153" t="n">
-        <v>6902000000</v>
-      </c>
-      <c r="F153" t="n">
-        <v>11398108182.78608</v>
-      </c>
-      <c r="G153" t="n">
-        <v>165.1421063863529</v>
-      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>page 15 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5879,7 +5769,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -5890,23 +5780,17 @@
       <c r="D154" t="n">
         <v>657355257.8779061</v>
       </c>
-      <c r="E154" t="n">
-        <v>2025000000</v>
-      </c>
-      <c r="F154" t="n">
-        <v>-1367644742.122094</v>
-      </c>
-      <c r="G154" t="n">
-        <v>-67.53801195664661</v>
-      </c>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>page 14 (OCR table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -5918,7 +5802,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>BFXS5XCH7N0Y05NIXW11</t>
+          <t>R4DHLH5KX7NMDO6YTPM4</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -5929,23 +5813,17 @@
       <c r="D155" t="n">
         <v>14694335353.459</v>
       </c>
-      <c r="E155" t="n">
-        <v>17600000</v>
-      </c>
-      <c r="F155" t="n">
-        <v>14676735353.459</v>
-      </c>
-      <c r="G155" t="n">
-        <v>83390.54178101705</v>
-      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>PDF non disponible</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>page 14 (OCR table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -6475,23 +6353,17 @@
       <c r="D169" t="n">
         <v>3097160515.81</v>
       </c>
-      <c r="E169" t="n">
-        <v>62000000</v>
-      </c>
-      <c r="F169" t="n">
-        <v>3035160515.81</v>
-      </c>
-      <c r="G169" t="n">
-        <v>4895.420186790322</v>
-      </c>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr">
         <is>
-          <t>ECART SIGNIFICATIF</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>page 142 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -7452,23 +7324,17 @@
       <c r="D198" t="n">
         <v>0.2453352409342637</v>
       </c>
-      <c r="E198" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="F198" t="n">
-        <v>0.0003352409342637086</v>
-      </c>
-      <c r="G198" t="n">
-        <v>0.1368330343933505</v>
-      </c>
+      <c r="E198" t="inlineStr"/>
+      <c r="F198" t="inlineStr"/>
+      <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>page 108 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -7491,23 +7357,17 @@
       <c r="D199" t="n">
         <v>0.2453352409342637</v>
       </c>
-      <c r="E199" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="F199" t="n">
-        <v>0.0003352409342637086</v>
-      </c>
-      <c r="G199" t="n">
-        <v>0.1368330343933505</v>
-      </c>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>page 108 (Qwen2.5-VL)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -7530,23 +7390,17 @@
       <c r="D200" t="n">
         <v>0.2470637829637899</v>
       </c>
-      <c r="E200" t="n">
-        <v>0.247</v>
-      </c>
-      <c r="F200" t="n">
-        <v>6.378296378994897e-05</v>
-      </c>
-      <c r="G200" t="n">
-        <v>0.02582306226313723</v>
-      </c>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>page 108 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -7570,22 +7424,22 @@
         <v>0.0965</v>
       </c>
       <c r="E201" t="n">
-        <v>0.0965</v>
+        <v>0.113</v>
       </c>
       <c r="F201" t="n">
-        <v>0</v>
+        <v>-0.0165</v>
       </c>
       <c r="G201" t="n">
-        <v>0</v>
+        <v>-14.60176991150442</v>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>ECART SIGNIFICATIF</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>page 110</t>
+          <t>page 131 (table)</t>
         </is>
       </c>
     </row>
@@ -7609,13 +7463,13 @@
         <v>1.2087</v>
       </c>
       <c r="E202" t="n">
-        <v>1</v>
+        <v>1.24</v>
       </c>
       <c r="F202" t="n">
-        <v>0.2087000000000001</v>
+        <v>-0.03129999999999988</v>
       </c>
       <c r="G202" t="n">
-        <v>20.87000000000001</v>
+        <v>-2.524193548387087</v>
       </c>
       <c r="H202" t="inlineStr">
         <is>
@@ -7624,7 +7478,7 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>page 54 (table)</t>
+          <t>page 130 (table)</t>
         </is>
       </c>
     </row>
@@ -7686,23 +7540,17 @@
       <c r="D204" t="n">
         <v>3868429342.22</v>
       </c>
-      <c r="E204" t="n">
-        <v>3869000000</v>
-      </c>
-      <c r="F204" t="n">
-        <v>-570657.7800002098</v>
-      </c>
-      <c r="G204" t="n">
-        <v>-0.01474949030757844</v>
-      </c>
+      <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr"/>
+      <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>page 108 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -7725,23 +7573,17 @@
       <c r="D205" t="n">
         <v>3868429342.22</v>
       </c>
-      <c r="E205" t="n">
-        <v>3869000000</v>
-      </c>
-      <c r="F205" t="n">
-        <v>-570657.7800002098</v>
-      </c>
-      <c r="G205" t="n">
-        <v>-0.01474949030757844</v>
-      </c>
+      <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr"/>
+      <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>page 108 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -7764,23 +7606,17 @@
       <c r="D206" t="n">
         <v>3895684875.02</v>
       </c>
-      <c r="E206" t="n">
-        <v>3896000000</v>
-      </c>
-      <c r="F206" t="n">
-        <v>-315124.9800000191</v>
-      </c>
-      <c r="G206" t="n">
-        <v>-0.008088423511294124</v>
-      </c>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
+      <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>page 108 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>
@@ -7803,23 +7639,17 @@
       <c r="D207" t="n">
         <v>15767931779.75</v>
       </c>
-      <c r="E207" t="n">
-        <v>15768000000</v>
-      </c>
-      <c r="F207" t="n">
-        <v>-68220.25</v>
-      </c>
-      <c r="G207" t="n">
-        <v>-0.0004326499873160832</v>
-      </c>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr"/>
+      <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Non trouvé dans le PDF</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>page 108 (table)</t>
+          <t>auto-extraction (KM1/OV1 regex)</t>
         </is>
       </c>
     </row>

</xml_diff>